<commit_message>
Fix Excel KPI data - all 3 metrics per market filled
</commit_message>
<xml_diff>
--- a/biweekly/2026-05-19/report.xlsx
+++ b/biweekly/2026-05-19/report.xlsx
@@ -93,12 +93,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002D6CDF"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="002D6CDF"/>
       </patternFill>
     </fill>
     <fill>
@@ -158,20 +158,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,7 +196,9 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -226,7 +232,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -244,8 +250,17 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -616,11 +631,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -655,7 +670,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1">
+    <row r="5" ht="55" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>🇮🇱 以色列</t>
@@ -668,12 +683,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>终端完成率 92%，库销比 2.7，出运正常。
-P145 大客户激励待审批。已预生产 500 台 P145，船期 6月10日。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="50" customHeight="1">
+          <t>终端完成率 92%，库销比 2.7，出运正常。P145 大客户激励待审批。
+已预生产 500 台 P145，船期 6月10日。需尽快补充终端库存。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>🇮🇹 意大利</t>
@@ -687,11 +702,11 @@
       <c r="C6" s="9" t="inlineStr">
         <is>
           <t>累计结算仅 1 台（H1 目标 3173 台），2500 台待 6 月结算。
-需尽快确认支持方案和 E2 价格以完成订单结算。终端库销比 4.5。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="50" customHeight="1">
+需尽快确认 E2 价格和法务主体资质以完成订单结算。终端库销比 4.5。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>🇵🇱 波兰</t>
@@ -705,11 +720,11 @@
       <c r="C7" s="6" t="inlineStr">
         <is>
           <t>终端完成率 9.3%，库销比 18.4（健康值 &lt;3）。
-积压超 600 台 MY2025 老库存，Q2 另有 2300 台到港。需协调清库方案。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="50" customHeight="1">
+积压超 600 台 MY2025 老库存，Q2 另有 2300 台到港。库存压力极大。需协调清库方案和周边市场转库。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>🇬🇷 希腊</t>
@@ -723,7 +738,7 @@
       <c r="C8" s="9" t="inlineStr">
         <is>
           <t>零结算、零出运。经销商库存仅 139 台。
-市场近乎停摆，总代不接受 FOB 价格。急需从意大利转库补货。</t>
+市场近乎停摆，急需补货。总代不接受最新 FOB 价格。正在协调从意大利转库补充终端。</t>
         </is>
       </c>
     </row>
@@ -736,9 +751,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -751,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -805,7 +820,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
           <t>希腊</t>
@@ -813,22 +828,21 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>致命</t>
+          <t>🔴 致命</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>市场完全停摆。结算和出运均为零，仅 139 台库存。
-总代不接受 P145/E245 的最新 FOB 价格。</t>
+          <t>市场完全停摆。结算和出运均为零，仅 139 台库存。总代不接受 P145/E245 最新 FOB。</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Q2 营收归零。经销商无车可卖。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="50" customHeight="1">
+          <t>Q2 营收归零。经销商无车可卖，渠道信心崩塌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
           <t>波兰</t>
@@ -836,22 +850,21 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>严重</t>
+          <t>🟠 严重</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>高库存积压 + 终端销售疲软。库销比 18.4。
-超 600 台 MY2025 老库存未清，Q2 将到港 2300 台。</t>
+          <t>高库存积压+终端销售疲软。库销比 18.4（目标 &lt;3）。超 600 台 MY2025 老库存，Q2 再进 2300 台。</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>25 年型亏损扩大。经销商现金流承压。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="50" customHeight="1">
+          <t>25 年型亏损扩大。库存资金占用恶化，经销商现金流承压。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
           <t>意大利</t>
@@ -859,22 +872,21 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>关注</t>
+          <t>🟡 关注</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>结算问题卡住全盘。仅结算 1 台（H1 目标 3173）。
-需 E2 底价和法务主体资质才能重启。</t>
+          <t>结算阻塞。仅 1 台结算（H1 目标 3173）。需 E2 底价+法务主体资质解锁 2500 台待结算。</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>定价/法务导致供应链断裂风险。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="50" customHeight="1">
+          <t>定价/法务问题导致供应链断裂。2500 台订单悬空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="22" t="inlineStr">
         <is>
           <t>以色列</t>
@@ -882,17 +894,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>可控</t>
+          <t>🟢 可控</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>大客户激励方案待审批。终端完成率 92%。</t>
+          <t>大客户激励待审批。终端完成率 92%，库销比 2.7。</t>
         </is>
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>影响 Q2 出运节奏，但风险可控。</t>
+          <t>影响 Q2 出运节奏，但整体可控。</t>
         </is>
       </c>
     </row>
@@ -928,12 +940,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>总代不接受 FOB → 价格高于预期 → P145/E245 定价超出市场承受力 → 市场由以色列总代管理 → 以色列总代将以色列市场的利润预期套用在希腊市场</t>
+          <t>总代不接受 FOB → 价格高于预期 → P145/E245 定价超出希腊市场承受力 → 希腊由以色列总代管理 → 以色列将本土利润预期套用在希腊</t>
         </is>
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>代理结构缺陷：希腊无独立总代，受以色列利润模型约束</t>
+          <t>代理结构缺陷：希腊无独立总代，利润模型不匹配当地市场</t>
         </is>
       </c>
     </row>
@@ -945,12 +957,12 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>库销比 18.4 → Q1 清库未启动 → 等待 MY2025→2026 折价政策 → 总部审批流程缓慢 → 缺乏车型年切换的标准操作流程（SOP）</t>
+          <t>库销比 18.4 → Q1 清库未启动 → MY2025→2026 折价政策等待审批 → 总部跨部门流程慢 → 缺乏标准化的车型年切换 SOP</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>缺乏生命周期管理机制，清库决策依赖逐次审批</t>
+          <t>缺乏生命周期管理机制，清库决策依赖逐次审批而非标准化流程</t>
         </is>
       </c>
     </row>
@@ -962,540 +974,540 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>仅 1 台结算 → 法务主体资质待批 → 涉及法务+财务+销售跨部门决策 → 原有金融工具切换时无备选方案 → 结算主渠道切换时缺乏应急预案</t>
+          <t>仅 1 台结算 → 法务主体资质待批 → 涉及法务+财务+销售跨部门决策 → 原金融工具切换时无备选方案 → 结算主渠道中断无应急</t>
         </is>
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>跨部门决策链断裂，无 contingency plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+          <t>跨部门决策链断裂，主渠道切换时缺乏 contingency plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>3. 对策与资源协调</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>行动项</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>截止日</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>负责人</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>所需资源</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="27" t="inlineStr">
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>意大利法务主体资质 — 完成跨部门审批，解锁结算通道</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>5月底</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D19" s="27" t="inlineStr">
         <is>
           <t>Justin + 法务</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E19" s="27" t="inlineStr">
         <is>
           <t>法务团队签批</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="27" t="inlineStr">
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>E2 底价 + 意大利一国一价 — 释放定价方案，重启 Q2 结算</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>5月底</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>Justin + 总部定价</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>总部定价审批</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="27" t="inlineStr">
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>波兰 MY2025 清库政策 — 发布折价方案，启动清库降低库销比</t>
-        </is>
-      </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>波兰 MY2025 清库政策 — 发布折价方案，阻止库销比恶化</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>5月内</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>LEO + 财务</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>财务折价授权</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="28" t="inlineStr">
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>意大利 Q2 大客户补贴 — 确认方案，推动 2500 台结算</t>
         </is>
       </c>
-      <c r="C21" s="28" t="inlineStr">
+      <c r="C22" s="28" t="inlineStr">
         <is>
           <t>6月初</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D22" s="28" t="inlineStr">
         <is>
           <t>孙百荷 + 总部</t>
         </is>
       </c>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="E22" s="28" t="inlineStr">
         <is>
           <t>预算授权</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="28" t="inlineStr">
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B23" s="28" t="inlineStr">
         <is>
           <t>以色列 P145 激励审批 — 完成大客户激励签批</t>
         </is>
       </c>
-      <c r="C22" s="28" t="inlineStr">
+      <c r="C23" s="28" t="inlineStr">
         <is>
           <t>下周</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>Justin + 总部</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
         <is>
           <t>相关部门签批</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="28" t="inlineStr">
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B24" s="28" t="inlineStr">
         <is>
           <t>希腊补货 — 从意大利调拨 130 台至希腊</t>
         </is>
       </c>
-      <c r="C23" s="28" t="inlineStr">
+      <c r="C24" s="28" t="inlineStr">
         <is>
           <t>5月23日</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D24" s="28" t="inlineStr">
         <is>
           <t>Rica + 物流</t>
         </is>
       </c>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="E24" s="28" t="inlineStr">
         <is>
           <t>转库协调</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>4. 跟进计划与标准化推广</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>优先级</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>任务</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>负责人</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>截止日</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>标准化产出</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="25" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>意大利法务主体</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>Justin</t>
         </is>
       </c>
-      <c r="D27" s="27" t="inlineStr">
+      <c r="D28" s="27" t="inlineStr">
         <is>
           <t>5月底</t>
         </is>
       </c>
-      <c r="E27" s="27" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>待决策</t>
         </is>
       </c>
-      <c r="F27" s="15" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>跨境法务主体设立 SOP</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="25" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>E2 底价释放</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>总部定价</t>
         </is>
       </c>
-      <c r="D28" s="27" t="inlineStr">
+      <c r="D29" s="27" t="inlineStr">
         <is>
           <t>5月底</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
         <is>
           <t>待发布</t>
         </is>
       </c>
-      <c r="F28" s="15" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="25" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>波兰清库政策</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>LEO</t>
         </is>
       </c>
-      <c r="D29" s="27" t="inlineStr">
+      <c r="D30" s="27" t="inlineStr">
         <is>
           <t>5月底</t>
         </is>
       </c>
-      <c r="E29" s="27" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>待发布</t>
         </is>
       </c>
-      <c r="F29" s="15" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>车型年切换 SOP</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="25" customHeight="1">
-      <c r="A30" s="29" t="inlineStr">
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="29" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>意大利大客户补贴</t>
         </is>
       </c>
-      <c r="C30" s="20" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>孙百荷</t>
         </is>
       </c>
-      <c r="D30" s="28" t="inlineStr">
+      <c r="D31" s="28" t="inlineStr">
         <is>
           <t>6月初</t>
         </is>
       </c>
-      <c r="E30" s="28" t="inlineStr">
+      <c r="E31" s="28" t="inlineStr">
         <is>
           <t>待审批</t>
         </is>
       </c>
-      <c r="F30" s="20" t="inlineStr">
+      <c r="F31" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="25" customHeight="1">
-      <c r="A31" s="29" t="inlineStr">
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>以色列 P145 激励</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>Justin</t>
         </is>
       </c>
-      <c r="D31" s="28" t="inlineStr">
+      <c r="D32" s="28" t="inlineStr">
         <is>
           <t>下周</t>
         </is>
       </c>
-      <c r="E31" s="28" t="inlineStr">
+      <c r="E32" s="28" t="inlineStr">
         <is>
           <t>待审批</t>
         </is>
       </c>
-      <c r="F31" s="20" t="inlineStr">
+      <c r="F32" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="25" customHeight="1">
-      <c r="A32" s="29" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="29" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>希腊结算完成</t>
         </is>
       </c>
-      <c r="C32" s="20" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>Rica</t>
         </is>
       </c>
-      <c r="D32" s="28" t="inlineStr">
+      <c r="D33" s="28" t="inlineStr">
         <is>
           <t>5月底</t>
         </is>
       </c>
-      <c r="E32" s="28" t="inlineStr">
+      <c r="E33" s="28" t="inlineStr">
         <is>
           <t>待推动</t>
         </is>
       </c>
-      <c r="F32" s="20" t="inlineStr">
+      <c r="F33" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="25" customHeight="1">
-      <c r="A33" s="29" t="inlineStr">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="29" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>希腊补货 130 台</t>
         </is>
       </c>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>Rica</t>
         </is>
       </c>
-      <c r="D33" s="28" t="inlineStr">
+      <c r="D34" s="28" t="inlineStr">
         <is>
           <t>5月23日</t>
         </is>
       </c>
-      <c r="E33" s="28" t="inlineStr">
+      <c r="E34" s="28" t="inlineStr">
         <is>
           <t>执行中</t>
         </is>
       </c>
-      <c r="F33" s="20" t="inlineStr">
+      <c r="F34" s="20" t="inlineStr">
         <is>
           <t>跨区域转库 SOP</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="25" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B34" s="23" t="inlineStr">
+      <c r="B35" s="23" t="inlineStr">
         <is>
           <t>波兰清库效果复盘</t>
         </is>
       </c>
-      <c r="C34" s="23" t="inlineStr">
+      <c r="C35" s="23" t="inlineStr">
         <is>
           <t>LEO</t>
         </is>
       </c>
-      <c r="D34" s="30" t="inlineStr">
+      <c r="D35" s="30" t="inlineStr">
         <is>
           <t>6月中</t>
         </is>
       </c>
-      <c r="E34" s="30" t="inlineStr">
+      <c r="E35" s="30" t="inlineStr">
         <is>
           <t>待启动</t>
         </is>
       </c>
-      <c r="F34" s="23" t="inlineStr">
+      <c r="F35" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="25" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B36" s="23" t="inlineStr">
         <is>
           <t>Launch Checklist 更新</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C36" s="23" t="inlineStr">
         <is>
           <t>全组</t>
         </is>
       </c>
-      <c r="D35" s="30" t="inlineStr">
+      <c r="D36" s="30" t="inlineStr">
         <is>
           <t>持续</t>
         </is>
       </c>
-      <c r="E35" s="30" t="inlineStr">
+      <c r="E36" s="30" t="inlineStr">
         <is>
           <t>进行中</t>
         </is>
       </c>
-      <c r="F35" s="23" t="inlineStr">
+      <c r="F36" s="23" t="inlineStr">
         <is>
           <t>Launch Checklist 模板</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>P0 = 本周必须完成（阻塞 Q2） · P1 = 本月完成 · P2 = 持续跟踪</t>
         </is>
@@ -1503,13 +1515,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A4:D4"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A26:F26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1522,18 +1534,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1565,586 +1574,521 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>结算 (台)</t>
+          <t>结算</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>结算 %</t>
+          <t>出运</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>出运 (台)</t>
+          <t>终端</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>出运 %</t>
+          <t>经销商库存</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>终端 (台)</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>终端 %</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>经销商库存 (台)</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
           <t>库销比</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>台 / 率</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>台 / 率</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>台 / 率</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>(台)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>意大利</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>1 / 0.04%</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>— / 121%</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>— / —</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="31" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>0 / 0%</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="inlineStr">
+        <is>
+          <t>— / 170%</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>— / 9.3%</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="inlineStr">
+        <is>
+          <t>600+</t>
+        </is>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>— / 31.4%</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>— / 38%</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>— / 92%</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>0 / 0%</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="inlineStr">
+        <is>
+          <t>0 / 0%</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="inlineStr">
+        <is>
+          <t>— / 31%</t>
+        </is>
+      </c>
+      <c r="E10" s="32" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>C大区合计</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>— / 14.3%</t>
+        </is>
+      </c>
+      <c r="C11" s="34" t="inlineStr">
+        <is>
+          <t>— / 89%</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>— / 47%</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>健康参考</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>— / &gt;50%</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>— / &gt;80%</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>— / &gt;80%</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>&lt;3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>2. 5-6月预测 &amp; H1 整体缺口分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>市场</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>H1 目标 (台)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>1-4月实际 (台)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>5-6月预测 (台)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>H1 缺口 (台)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>缺口 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="n">
+        <v>3173</v>
+      </c>
+      <c r="C16" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>0.04%</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D16" s="31" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E16" s="31" t="n">
+        <v>-672</v>
+      </c>
+      <c r="F16" s="31" t="inlineStr">
+        <is>
+          <t>-21.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>121%</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="C17" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="E17" s="32" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>-80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>波兰</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D19" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="32" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>170%</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>600+</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="n">
-        <v>18.4</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>以色列</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>31.4%</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>92%</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>2.7</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>希腊</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>31%</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>139</v>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>-100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="34" t="inlineStr">
         <is>
           <t>C大区合计</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-      <c r="D10" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="31" t="inlineStr">
-        <is>
-          <t>89%</t>
-        </is>
-      </c>
-      <c r="F10" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="31" t="inlineStr">
-        <is>
-          <t>47%</t>
-        </is>
-      </c>
-      <c r="H10" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>健康参考</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
-        <is>
-          <t>&gt;50%</t>
-        </is>
-      </c>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>&gt;80%</t>
-        </is>
-      </c>
-      <c r="F11" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>&gt;80%</t>
-        </is>
-      </c>
-      <c r="H11" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="24" t="inlineStr">
-        <is>
-          <t>&lt;3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2. 5-6月预测 &amp; H1 整体缺口分析</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>市场</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>H1 目标 (台)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>1-4月实际 (台)</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>5-6月预测 (台)</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>H1 缺口 (台)</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>缺口 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>意大利</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>3173</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>-672</v>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>-21.2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>波兰</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>-80%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>以色列</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>希腊</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>-100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="31" t="inlineStr">
-        <is>
-          <t>C大区合计</t>
-        </is>
-      </c>
-      <c r="B19" s="31" t="n">
+      <c r="B21" s="34" t="n">
         <v>9282</v>
       </c>
-      <c r="C19" s="31" t="n">
+      <c r="C21" s="34" t="n">
         <v>1327</v>
       </c>
-      <c r="D19" s="31" t="n">
+      <c r="D21" s="34" t="n">
         <v>4853</v>
       </c>
-      <c r="E19" s="31" t="n">
+      <c r="E21" s="34" t="n">
         <v>-3102</v>
       </c>
-      <c r="F19" s="31" t="inlineStr">
+      <c r="F21" s="34" t="inlineStr">
         <is>
           <t>-33.4%</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>3. H1 缺口总结 — 按严重程度排序</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>缺口类型</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>数据</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>分析</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="27" t="inlineStr">
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>致命 — 终端缺口</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>-4778 台 (-38.2%)</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>终端是经销商的命脉。近 5000 台缺口意味着 Q3 需要大幅度追赶。波兰和希腊拖累最大。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>-4,778 台 (-38.2%)</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>终端是经销商的生命线。近 5000 台缺口意味着 Q3 需大幅追赶。波兰（完成率 9.3%）和希腊（31%）拖累最大，是 H1 最核心的交付风险。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="35" t="inlineStr">
         <is>
           <t>🟠</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>严重 — 结算缺口</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>-3102 台 (-33.4%)</t>
-        </is>
-      </c>
-      <c r="D24" s="17" t="inlineStr">
-        <is>
-          <t>终端疲软导致结算不畅，现金回流受阻，供应链面临断裂风险。波兰最严重（-80%）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>-3,102 台 (-33.4%)</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>终端疲软直接导致结算不畅，现金回流受阻，供应链面临停顿风险。波兰最严重（缺口-80%），意大利次之（-21.2%）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>可控 — 出运缺口</t>
         </is>
       </c>
-      <c r="C25" s="24" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>-352 台 (-3.2%)</t>
         </is>
       </c>
-      <c r="D25" s="23" t="inlineStr">
-        <is>
-          <t>非核心矛盾。波兰出运超目标对冲了希腊零出运。希腊可通过转库补货解决。</t>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>非核心矛盾。波兰出运超目标（+350 台）对冲了希腊零出运，整体偏差仅 3.2%。希腊零出运可通过意大利转库补货解决。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A21:J21"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>